<commit_message>
Added the deviation penalty column to the example input files.
Added the deviation penalty column to the example input files.
</commit_message>
<xml_diff>
--- a/input_data/demo_model.xlsx
+++ b/input_data/demo_model.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dsdennis\HOPE\Predicer\input_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126EFFD4-1C7C-44ED-B784-97D3C87E86E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46B8C23A-0DC2-43C6-ACA4-F6422450FE6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="796" firstSheet="7" activeTab="14" xr2:uid="{788BFBD1-D930-4535-8A91-D85C56924796}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="132">
   <si>
     <t>node</t>
   </si>
@@ -454,6 +454,9 @@
   </si>
   <si>
     <t>inflow</t>
+  </si>
+  <si>
+    <t>deviation_penalty</t>
   </si>
 </sst>
 </file>
@@ -5897,13 +5900,13 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{076D8023-527F-4386-8A27-2EF08439356E}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>126</v>
       </c>
@@ -5921,6 +5924,9 @@
       </c>
       <c r="F1" t="s">
         <v>130</v>
+      </c>
+      <c r="G1" t="s">
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>